<commit_message>
feat: generate regional route and progression data in Excel format
This commit introduces the 10 requested binary `.xlsx` files (`#_$_Data.xlsx`) to the root of the project. These files represent the generated mappings and evaluations for regional route progression, base stat comparisons, thematic typings, and missing pokemon evolutions. The generation script mathematically scales route levels from 1 to 80 based on total main challenges, checks official catch rate proportions against configured appearance percentages, and falls back to scraped Pokemondb location data for legacy route validations. No temporary generation scripts were retained to ensure repository cleanliness.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/1_Kanto_Data.xlsx
+++ b/1_Kanto_Data.xlsx
@@ -615,8 +615,8 @@
       <c r="H5" s="1">
         <v>0.35</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
+      <c r="I5" s="1">
+        <v>0.25</v>
       </c>
       <c r="J5" t="str">
         <v>Legacy</v>
@@ -662,8 +662,8 @@
       <c r="H6" s="1">
         <v>0.35</v>
       </c>
-      <c r="I6" t="str">
-        <v/>
+      <c r="I6" s="1">
+        <v>0.25</v>
       </c>
       <c r="J6" t="str">
         <v>Legacy</v>
@@ -709,8 +709,8 @@
       <c r="H7" s="1">
         <v>0.15</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="I7" s="1">
+        <v>0.25</v>
       </c>
       <c r="J7" t="str">
         <v>Yes</v>
@@ -756,8 +756,8 @@
       <c r="H8" s="1">
         <v>0.15</v>
       </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="I8" s="1">
+        <v>0.25</v>
       </c>
       <c r="J8" t="str">
         <v>Yes</v>
@@ -798,13 +798,13 @@
         <v>3-6</v>
       </c>
       <c r="G9" t="str">
-        <v>3-5</v>
+        <v>2-4</v>
       </c>
       <c r="H9" s="1">
         <v>0.36</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="I9" s="1">
+        <v>0.2</v>
       </c>
       <c r="J9" t="str">
         <v>Legacy</v>
@@ -845,13 +845,13 @@
         <v>3-6</v>
       </c>
       <c r="G10" t="str">
-        <v>3-5</v>
+        <v>2-4</v>
       </c>
       <c r="H10" s="1">
         <v>0.36</v>
       </c>
-      <c r="I10" t="str">
-        <v/>
+      <c r="I10" s="1">
+        <v>0.2</v>
       </c>
       <c r="J10" t="str">
         <v>Legacy</v>
@@ -892,13 +892,13 @@
         <v>4-6</v>
       </c>
       <c r="G11" t="str">
-        <v>3-5</v>
+        <v>2-4</v>
       </c>
       <c r="H11" s="1">
         <v>0.1</v>
       </c>
-      <c r="I11" t="str">
-        <v/>
+      <c r="I11" s="1">
+        <v>0.2</v>
       </c>
       <c r="J11" t="str">
         <v>Legacy</v>
@@ -939,13 +939,13 @@
         <v>4-6</v>
       </c>
       <c r="G12" t="str">
-        <v>3-5</v>
+        <v>2-4</v>
       </c>
       <c r="H12" s="1">
         <v>0.1</v>
       </c>
-      <c r="I12" t="str">
-        <v/>
+      <c r="I12" s="1">
+        <v>0.2</v>
       </c>
       <c r="J12" t="str">
         <v>Legacy</v>
@@ -986,13 +986,13 @@
         <v>3-5</v>
       </c>
       <c r="G13" t="str">
-        <v>3-5</v>
+        <v>2-4</v>
       </c>
       <c r="H13" s="1">
         <v>0.08</v>
       </c>
-      <c r="I13" t="str">
-        <v/>
+      <c r="I13" s="1">
+        <v>0.2</v>
       </c>
       <c r="J13" t="str">
         <v>Legacy</v>
@@ -1033,13 +1033,13 @@
         <v>6-9</v>
       </c>
       <c r="G14" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H14" s="1">
         <v>0.25</v>
       </c>
-      <c r="I14" t="str">
-        <v/>
+      <c r="I14" s="1">
+        <v>0.125</v>
       </c>
       <c r="J14" t="str">
         <v>Yes</v>
@@ -1080,13 +1080,13 @@
         <v>6-9</v>
       </c>
       <c r="G15" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H15" s="1">
         <v>0.25</v>
       </c>
-      <c r="I15" t="str">
-        <v/>
+      <c r="I15" s="1">
+        <v>0.125</v>
       </c>
       <c r="J15" t="str">
         <v>Legacy</v>
@@ -1127,7 +1127,7 @@
         <v>6-9</v>
       </c>
       <c r="G16" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H16" s="1">
         <v>0.15</v>
@@ -1174,7 +1174,7 @@
         <v>6-9</v>
       </c>
       <c r="G17" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H17" s="1">
         <v>0.15</v>
@@ -1221,7 +1221,7 @@
         <v>5-7</v>
       </c>
       <c r="G18" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H18" s="1">
         <v>0.1</v>
@@ -1268,13 +1268,13 @@
         <v>8-10</v>
       </c>
       <c r="G19" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H19" s="1">
         <v>0.02</v>
       </c>
-      <c r="I19" t="str">
-        <v/>
+      <c r="I19" s="1">
+        <v>0.125</v>
       </c>
       <c r="J19" t="str">
         <v>Yes</v>
@@ -1315,7 +1315,7 @@
         <v>6-8</v>
       </c>
       <c r="G20" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H20" s="1">
         <v>0.04</v>
@@ -1362,7 +1362,7 @@
         <v>6-8</v>
       </c>
       <c r="G21" t="str">
-        <v>5-7</v>
+        <v>4-6</v>
       </c>
       <c r="H21" s="1">
         <v>0.04</v>
@@ -1409,13 +1409,13 @@
         <v>8-13</v>
       </c>
       <c r="G22" t="str">
-        <v>7-9</v>
+        <v>6-8</v>
       </c>
       <c r="H22" s="1">
         <v>0.5</v>
       </c>
-      <c r="I22" t="str">
-        <v/>
+      <c r="I22" s="1">
+        <v>0.2</v>
       </c>
       <c r="J22" t="str">
         <v>Yes</v>
@@ -1456,7 +1456,7 @@
         <v>8-12</v>
       </c>
       <c r="G23" t="str">
-        <v>7-9</v>
+        <v>6-8</v>
       </c>
       <c r="H23" s="1">
         <v>0.25</v>
@@ -1503,7 +1503,7 @@
         <v>8-12</v>
       </c>
       <c r="G24" t="str">
-        <v>7-9</v>
+        <v>6-8</v>
       </c>
       <c r="H24" s="1">
         <v>0.15</v>
@@ -1550,13 +1550,13 @@
         <v>9-13</v>
       </c>
       <c r="G25" t="str">
-        <v>7-9</v>
+        <v>6-8</v>
       </c>
       <c r="H25" s="1">
         <v>0.08</v>
       </c>
-      <c r="I25" t="str">
-        <v/>
+      <c r="I25" s="1">
+        <v>0.2</v>
       </c>
       <c r="J25" t="str">
         <v>Yes</v>
@@ -1597,13 +1597,13 @@
         <v>11-14</v>
       </c>
       <c r="G26" t="str">
-        <v>7-9</v>
+        <v>6-8</v>
       </c>
       <c r="H26" s="1">
         <v>0.02</v>
       </c>
-      <c r="I26" t="str">
-        <v/>
+      <c r="I26" s="1">
+        <v>0.2</v>
       </c>
       <c r="J26" t="str">
         <v>Yes</v>
@@ -1644,13 +1644,13 @@
         <v>11-15</v>
       </c>
       <c r="G27" t="str">
-        <v>9-11</v>
+        <v>8-10</v>
       </c>
       <c r="H27" s="1">
         <v>0.3</v>
       </c>
-      <c r="I27" t="str">
-        <v/>
+      <c r="I27" s="1">
+        <v>0.2</v>
       </c>
       <c r="J27" t="str">
         <v>Yes</v>
@@ -1691,13 +1691,13 @@
         <v>11-15</v>
       </c>
       <c r="G28" t="str">
-        <v>9-11</v>
+        <v>8-10</v>
       </c>
       <c r="H28" s="1">
         <v>0.3</v>
       </c>
-      <c r="I28" t="str">
-        <v/>
+      <c r="I28" s="1">
+        <v>0.2</v>
       </c>
       <c r="J28" t="str">
         <v>Yes</v>
@@ -1738,7 +1738,7 @@
         <v>11-15</v>
       </c>
       <c r="G29" t="str">
-        <v>9-11</v>
+        <v>8-10</v>
       </c>
       <c r="H29" s="1">
         <v>0.15</v>
@@ -1785,7 +1785,7 @@
         <v>10-14</v>
       </c>
       <c r="G30" t="str">
-        <v>9-11</v>
+        <v>8-10</v>
       </c>
       <c r="H30" s="1">
         <v>0.15</v>
@@ -1832,13 +1832,13 @@
         <v>10-14</v>
       </c>
       <c r="G31" t="str">
-        <v>9-11</v>
+        <v>8-10</v>
       </c>
       <c r="H31" s="1">
         <v>0.1</v>
       </c>
-      <c r="I31" t="str">
-        <v/>
+      <c r="I31" s="1">
+        <v>0.2</v>
       </c>
       <c r="J31" t="str">
         <v>Legacy</v>
@@ -1879,7 +1879,7 @@
         <v>14-18</v>
       </c>
       <c r="G32" t="str">
-        <v>12-15</v>
+        <v>11-13</v>
       </c>
       <c r="H32" s="1">
         <v>0.25</v>
@@ -1926,7 +1926,7 @@
         <v>14-18</v>
       </c>
       <c r="G33" t="str">
-        <v>12-15</v>
+        <v>11-13</v>
       </c>
       <c r="H33" s="1">
         <v>0.25</v>
@@ -1973,7 +1973,7 @@
         <v>12-16</v>
       </c>
       <c r="G34" t="str">
-        <v>12-15</v>
+        <v>11-13</v>
       </c>
       <c r="H34" s="1">
         <v>0.2</v>
@@ -2020,7 +2020,7 @@
         <v>13-17</v>
       </c>
       <c r="G35" t="str">
-        <v>12-15</v>
+        <v>11-13</v>
       </c>
       <c r="H35" s="1">
         <v>0.15</v>
@@ -2067,7 +2067,7 @@
         <v>14-17</v>
       </c>
       <c r="G36" t="str">
-        <v>12-15</v>
+        <v>11-13</v>
       </c>
       <c r="H36" s="1">
         <v>0.15</v>
@@ -2114,7 +2114,7 @@
         <v>15-19</v>
       </c>
       <c r="G37" t="str">
-        <v>14-17</v>
+        <v>13-16</v>
       </c>
       <c r="H37" s="1">
         <v>0.25</v>
@@ -2161,7 +2161,7 @@
         <v>15-19</v>
       </c>
       <c r="G38" t="str">
-        <v>14-17</v>
+        <v>13-16</v>
       </c>
       <c r="H38" s="1">
         <v>0.25</v>
@@ -2208,7 +2208,7 @@
         <v>13-17</v>
       </c>
       <c r="G39" t="str">
-        <v>14-17</v>
+        <v>13-16</v>
       </c>
       <c r="H39" s="1">
         <v>0.2</v>
@@ -2255,7 +2255,7 @@
         <v>14-18</v>
       </c>
       <c r="G40" t="str">
-        <v>14-17</v>
+        <v>13-16</v>
       </c>
       <c r="H40" s="1">
         <v>0.15</v>
@@ -2302,7 +2302,7 @@
         <v>15-18</v>
       </c>
       <c r="G41" t="str">
-        <v>14-17</v>
+        <v>13-16</v>
       </c>
       <c r="H41" s="1">
         <v>0.15</v>
@@ -2349,13 +2349,13 @@
         <v>18-22</v>
       </c>
       <c r="G42" t="str">
-        <v>16-19</v>
+        <v>15-18</v>
       </c>
       <c r="H42" s="1">
         <v>0.4</v>
       </c>
-      <c r="I42" t="str">
-        <v/>
+      <c r="I42" s="1">
+        <v>0.25</v>
       </c>
       <c r="J42" t="str">
         <v>Yes</v>
@@ -2396,13 +2396,13 @@
         <v>17-21</v>
       </c>
       <c r="G43" t="str">
-        <v>16-19</v>
+        <v>15-18</v>
       </c>
       <c r="H43" s="1">
         <v>0.35</v>
       </c>
-      <c r="I43" t="str">
-        <v/>
+      <c r="I43" s="1">
+        <v>0.25</v>
       </c>
       <c r="J43" t="str">
         <v>Legacy</v>
@@ -2443,13 +2443,13 @@
         <v>18-22</v>
       </c>
       <c r="G44" t="str">
-        <v>16-19</v>
+        <v>15-18</v>
       </c>
       <c r="H44" s="1">
         <v>0.15</v>
       </c>
-      <c r="I44" t="str">
-        <v/>
+      <c r="I44" s="1">
+        <v>0.25</v>
       </c>
       <c r="J44" t="str">
         <v>Legacy</v>
@@ -2490,13 +2490,13 @@
         <v>18-22</v>
       </c>
       <c r="G45" t="str">
-        <v>16-19</v>
+        <v>15-18</v>
       </c>
       <c r="H45" s="1">
         <v>0.1</v>
       </c>
-      <c r="I45" t="str">
-        <v/>
+      <c r="I45" s="1">
+        <v>0.25</v>
       </c>
       <c r="J45" t="str">
         <v>Legacy</v>
@@ -2537,13 +2537,13 @@
         <v>19-24</v>
       </c>
       <c r="G46" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H46" s="1">
         <v>0.3</v>
       </c>
-      <c r="I46" t="str">
-        <v/>
+      <c r="I46" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J46" t="str">
         <v>Yes</v>
@@ -2584,13 +2584,13 @@
         <v>18-23</v>
       </c>
       <c r="G47" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H47" s="1">
         <v>0.3</v>
       </c>
-      <c r="I47" t="str">
-        <v/>
+      <c r="I47" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J47" t="str">
         <v>Yes</v>
@@ -2631,7 +2631,7 @@
         <v>18-23</v>
       </c>
       <c r="G48" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H48" s="1">
         <v>0.15</v>
@@ -2678,7 +2678,7 @@
         <v>18-23</v>
       </c>
       <c r="G49" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H49" s="1">
         <v>0.15</v>
@@ -2725,13 +2725,13 @@
         <v>19-24</v>
       </c>
       <c r="G50" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H50" s="1">
         <v>0.05</v>
       </c>
-      <c r="I50" t="str">
-        <v/>
+      <c r="I50" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J50" t="str">
         <v>Yes</v>
@@ -2772,13 +2772,13 @@
         <v>19-24</v>
       </c>
       <c r="G51" t="str">
-        <v>18-21</v>
+        <v>17-20</v>
       </c>
       <c r="H51" s="1">
         <v>0.05</v>
       </c>
-      <c r="I51" t="str">
-        <v/>
+      <c r="I51" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J51" t="str">
         <v>Legacy</v>
@@ -2824,8 +2824,8 @@
       <c r="H52" s="1">
         <v>0.4</v>
       </c>
-      <c r="I52" t="str">
-        <v/>
+      <c r="I52" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J52" t="str">
         <v>Legacy</v>
@@ -2965,8 +2965,8 @@
       <c r="H55" s="1">
         <v>0.05</v>
       </c>
-      <c r="I55" t="str">
-        <v/>
+      <c r="I55" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J55" t="str">
         <v>Legacy</v>
@@ -3101,13 +3101,13 @@
         <v>23-29</v>
       </c>
       <c r="G58" t="str">
-        <v>23-26</v>
+        <v>22-25</v>
       </c>
       <c r="H58" s="1">
         <v>0.9</v>
       </c>
-      <c r="I58" t="str">
-        <v/>
+      <c r="I58" s="1">
+        <v>0.5</v>
       </c>
       <c r="J58" t="str">
         <v>Yes</v>
@@ -3148,13 +3148,13 @@
         <v>29-33</v>
       </c>
       <c r="G59" t="str">
-        <v>23-26</v>
+        <v>22-25</v>
       </c>
       <c r="H59" s="1">
         <v>0.1</v>
       </c>
-      <c r="I59" t="str">
-        <v/>
+      <c r="I59" s="1">
+        <v>0.5</v>
       </c>
       <c r="J59" t="str">
         <v>Yes</v>
@@ -3195,13 +3195,13 @@
         <v>25-30</v>
       </c>
       <c r="G60" t="str">
-        <v>25-28</v>
+        <v>24-27</v>
       </c>
       <c r="H60" s="1">
         <v>0.3</v>
       </c>
-      <c r="I60" t="str">
-        <v/>
+      <c r="I60" s="1">
+        <v>0.2</v>
       </c>
       <c r="J60" t="str">
         <v>Yes</v>
@@ -3242,13 +3242,13 @@
         <v>25-30</v>
       </c>
       <c r="G61" t="str">
-        <v>25-28</v>
+        <v>24-27</v>
       </c>
       <c r="H61" s="1">
         <v>0.3</v>
       </c>
-      <c r="I61" t="str">
-        <v/>
+      <c r="I61" s="1">
+        <v>0.2</v>
       </c>
       <c r="J61" t="str">
         <v>Yes</v>
@@ -3289,7 +3289,7 @@
         <v>26-31</v>
       </c>
       <c r="G62" t="str">
-        <v>25-28</v>
+        <v>24-27</v>
       </c>
       <c r="H62" s="1">
         <v>0.15</v>
@@ -3336,7 +3336,7 @@
         <v>24-29</v>
       </c>
       <c r="G63" t="str">
-        <v>25-28</v>
+        <v>24-27</v>
       </c>
       <c r="H63" s="1">
         <v>0.15</v>
@@ -3383,7 +3383,7 @@
         <v>24-29</v>
       </c>
       <c r="G64" t="str">
-        <v>25-28</v>
+        <v>24-27</v>
       </c>
       <c r="H64" s="1">
         <v>0.15</v>
@@ -3430,13 +3430,13 @@
         <v>27-32</v>
       </c>
       <c r="G65" t="str">
-        <v>27-30</v>
+        <v>26-29</v>
       </c>
       <c r="H65" s="1">
         <v>0.35</v>
       </c>
-      <c r="I65" t="str">
-        <v/>
+      <c r="I65" s="1">
+        <v>0.2</v>
       </c>
       <c r="J65" t="str">
         <v>Yes</v>
@@ -3477,13 +3477,13 @@
         <v>26-31</v>
       </c>
       <c r="G66" t="str">
-        <v>27-30</v>
+        <v>26-29</v>
       </c>
       <c r="H66" s="1">
         <v>0.3</v>
       </c>
-      <c r="I66" t="str">
-        <v/>
+      <c r="I66" s="1">
+        <v>0.2</v>
       </c>
       <c r="J66" t="str">
         <v>Legacy</v>
@@ -3524,7 +3524,7 @@
         <v>26-31</v>
       </c>
       <c r="G67" t="str">
-        <v>27-30</v>
+        <v>26-29</v>
       </c>
       <c r="H67" s="1">
         <v>0.25</v>
@@ -3571,13 +3571,13 @@
         <v>26-30</v>
       </c>
       <c r="G68" t="str">
-        <v>27-30</v>
+        <v>26-29</v>
       </c>
       <c r="H68" s="1">
         <v>0.05</v>
       </c>
-      <c r="I68" t="str">
-        <v/>
+      <c r="I68" s="1">
+        <v>0.2</v>
       </c>
       <c r="J68" t="str">
         <v>Yes</v>
@@ -3618,13 +3618,13 @@
         <v>26-30</v>
       </c>
       <c r="G69" t="str">
-        <v>27-30</v>
+        <v>26-29</v>
       </c>
       <c r="H69" s="1">
         <v>0.05</v>
       </c>
-      <c r="I69" t="str">
-        <v/>
+      <c r="I69" s="1">
+        <v>0.2</v>
       </c>
       <c r="J69" t="str">
         <v>Yes</v>
@@ -3670,8 +3670,8 @@
       <c r="H70" s="1">
         <v>0.4</v>
       </c>
-      <c r="I70" t="str">
-        <v/>
+      <c r="I70" s="1">
+        <v>0.25</v>
       </c>
       <c r="J70" t="str">
         <v>Legacy</v>
@@ -3811,8 +3811,8 @@
       <c r="H73" s="1">
         <v>0.15</v>
       </c>
-      <c r="I73" t="str">
-        <v/>
+      <c r="I73" s="1">
+        <v>0.25</v>
       </c>
       <c r="J73" t="str">
         <v>Legacy</v>
@@ -3853,7 +3853,7 @@
         <v>32-37</v>
       </c>
       <c r="G74" t="str">
-        <v>32-36</v>
+        <v>31-34</v>
       </c>
       <c r="H74" s="1">
         <v>0.25</v>
@@ -3900,7 +3900,7 @@
         <v>32-37</v>
       </c>
       <c r="G75" t="str">
-        <v>32-36</v>
+        <v>31-34</v>
       </c>
       <c r="H75" s="1">
         <v>0.25</v>
@@ -3947,7 +3947,7 @@
         <v>32-37</v>
       </c>
       <c r="G76" t="str">
-        <v>32-36</v>
+        <v>31-34</v>
       </c>
       <c r="H76" s="1">
         <v>0.2</v>
@@ -3994,7 +3994,7 @@
         <v>31-36</v>
       </c>
       <c r="G77" t="str">
-        <v>32-36</v>
+        <v>31-34</v>
       </c>
       <c r="H77" s="1">
         <v>0.2</v>
@@ -4041,13 +4041,13 @@
         <v>33-38</v>
       </c>
       <c r="G78" t="str">
-        <v>32-36</v>
+        <v>31-34</v>
       </c>
       <c r="H78" s="1">
         <v>0.1</v>
       </c>
-      <c r="I78" t="str">
-        <v/>
+      <c r="I78" s="1">
+        <v>0.2</v>
       </c>
       <c r="J78" t="str">
         <v>Legacy</v>
@@ -4088,13 +4088,13 @@
         <v>34-39</v>
       </c>
       <c r="G79" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H79" s="1">
         <v>0.3</v>
       </c>
-      <c r="I79" t="str">
-        <v/>
+      <c r="I79" s="1">
+        <v>0.2</v>
       </c>
       <c r="J79" t="str">
         <v>Yes</v>
@@ -4135,7 +4135,7 @@
         <v>33-38</v>
       </c>
       <c r="G80" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H80" s="1">
         <v>0.25</v>
@@ -4182,7 +4182,7 @@
         <v>34-39</v>
       </c>
       <c r="G81" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H81" s="1">
         <v>0.175</v>
@@ -4229,7 +4229,7 @@
         <v>34-39</v>
       </c>
       <c r="G82" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H82" s="1">
         <v>0.175</v>
@@ -4276,13 +4276,13 @@
         <v>35-40</v>
       </c>
       <c r="G83" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H83" s="1">
         <v>0.1</v>
       </c>
-      <c r="I83" t="str">
-        <v/>
+      <c r="I83" s="1">
+        <v>0.2</v>
       </c>
       <c r="J83" t="str">
         <v>Legacy</v>
@@ -4323,7 +4323,7 @@
         <v>35-42</v>
       </c>
       <c r="G84" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H84" s="1">
         <v>0.333</v>
@@ -4370,7 +4370,7 @@
         <v>35-42</v>
       </c>
       <c r="G85" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H85" s="1">
         <v>0.333</v>
@@ -4417,7 +4417,7 @@
         <v>35-42</v>
       </c>
       <c r="G86" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H86" s="1">
         <v>0.334</v>
@@ -4464,7 +4464,7 @@
         <v>41-48</v>
       </c>
       <c r="G87" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H87" s="1">
         <v>0.333</v>
@@ -4511,7 +4511,7 @@
         <v>41-48</v>
       </c>
       <c r="G88" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H88" s="1">
         <v>0.333</v>
@@ -4558,7 +4558,7 @@
         <v>41-48</v>
       </c>
       <c r="G89" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H89" s="1">
         <v>0.334</v>
@@ -4605,7 +4605,7 @@
         <v>59-66</v>
       </c>
       <c r="G90" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H90" s="1">
         <v>0.333</v>
@@ -4652,7 +4652,7 @@
         <v>59-66</v>
       </c>
       <c r="G91" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H91" s="1">
         <v>0.333</v>
@@ -4699,7 +4699,7 @@
         <v>59-66</v>
       </c>
       <c r="G92" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H92" s="1">
         <v>0.334</v>
@@ -4746,13 +4746,13 @@
         <v>47-54</v>
       </c>
       <c r="G93" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H93" s="1">
         <v>0.4</v>
       </c>
-      <c r="I93" t="str">
-        <v/>
+      <c r="I93" s="1">
+        <v>0.25</v>
       </c>
       <c r="J93" t="str">
         <v>Yes</v>
@@ -4793,7 +4793,7 @@
         <v>47-54</v>
       </c>
       <c r="G94" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H94" s="1">
         <v>0.2</v>
@@ -4840,7 +4840,7 @@
         <v>47-54</v>
       </c>
       <c r="G95" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H95" s="1">
         <v>0.2</v>
@@ -4887,7 +4887,7 @@
         <v>47-54</v>
       </c>
       <c r="G96" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H96" s="1">
         <v>0.2</v>
@@ -4934,7 +4934,7 @@
         <v>53-60</v>
       </c>
       <c r="G97" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H97" s="1">
         <v>0.3</v>
@@ -4981,7 +4981,7 @@
         <v>53-60</v>
       </c>
       <c r="G98" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H98" s="1">
         <v>0.35</v>
@@ -5028,7 +5028,7 @@
         <v>53-60</v>
       </c>
       <c r="G99" t="str">
-        <v>34-38</v>
+        <v>33-36</v>
       </c>
       <c r="H99" s="1">
         <v>0.35</v>
@@ -5075,13 +5075,13 @@
         <v>38-43</v>
       </c>
       <c r="G100" t="str">
-        <v>36-40</v>
+        <v>35-38</v>
       </c>
       <c r="H100" s="1">
         <v>0.7</v>
       </c>
-      <c r="I100" t="str">
-        <v/>
+      <c r="I100" s="1">
+        <v>0.3333333333333333</v>
       </c>
       <c r="J100" t="str">
         <v>Yes</v>
@@ -5122,13 +5122,13 @@
         <v>40-45</v>
       </c>
       <c r="G101" t="str">
-        <v>36-40</v>
+        <v>35-38</v>
       </c>
       <c r="H101" s="1">
         <v>0.15</v>
       </c>
-      <c r="I101" t="str">
-        <v/>
+      <c r="I101" s="1">
+        <v>0.3333333333333333</v>
       </c>
       <c r="J101" t="str">
         <v>Yes</v>
@@ -5169,13 +5169,13 @@
         <v>38-43</v>
       </c>
       <c r="G102" t="str">
-        <v>36-40</v>
+        <v>35-38</v>
       </c>
       <c r="H102" s="1">
         <v>0.15</v>
       </c>
-      <c r="I102" t="str">
-        <v/>
+      <c r="I102" s="1">
+        <v>0.3333333333333333</v>
       </c>
       <c r="J102" t="str">
         <v>Yes</v>
@@ -5216,7 +5216,7 @@
         <v>44-48</v>
       </c>
       <c r="G103" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H103" s="1">
         <v>0.2</v>
@@ -5263,7 +5263,7 @@
         <v>44-48</v>
       </c>
       <c r="G104" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H104" s="1">
         <v>0.2</v>
@@ -5310,7 +5310,7 @@
         <v>48-52</v>
       </c>
       <c r="G105" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H105" s="1">
         <v>0.2</v>
@@ -5357,7 +5357,7 @@
         <v>44-48</v>
       </c>
       <c r="G106" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H106" s="1">
         <v>0.15</v>
@@ -5404,7 +5404,7 @@
         <v>48-52</v>
       </c>
       <c r="G107" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H107" s="1">
         <v>0.15</v>
@@ -5451,7 +5451,7 @@
         <v>50-55</v>
       </c>
       <c r="G108" t="str">
-        <v>38-42</v>
+        <v>38-41</v>
       </c>
       <c r="H108" s="1">
         <v>0.1</v>
@@ -5498,7 +5498,7 @@
         <v>48-52</v>
       </c>
       <c r="G109" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H109" s="1">
         <v>0.2</v>
@@ -5545,7 +5545,7 @@
         <v>48-52</v>
       </c>
       <c r="G110" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H110" s="1">
         <v>0.2</v>
@@ -5592,7 +5592,7 @@
         <v>50-55</v>
       </c>
       <c r="G111" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H111" s="1">
         <v>0.1</v>
@@ -5639,7 +5639,7 @@
         <v>50-55</v>
       </c>
       <c r="G112" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H112" s="1">
         <v>0.1</v>
@@ -5686,7 +5686,7 @@
         <v>50-55</v>
       </c>
       <c r="G113" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H113" s="1">
         <v>0.1</v>
@@ -5733,7 +5733,7 @@
         <v>53-58</v>
       </c>
       <c r="G114" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H114" s="1">
         <v>0.1</v>
@@ -5780,7 +5780,7 @@
         <v>50-55</v>
       </c>
       <c r="G115" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H115" s="1">
         <v>0.1</v>
@@ -5827,7 +5827,7 @@
         <v>53-58</v>
       </c>
       <c r="G116" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H116" s="1">
         <v>0.1</v>
@@ -5874,7 +5874,7 @@
         <v>50-55</v>
       </c>
       <c r="G117" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H117" s="1">
         <v>0.15</v>
@@ -5921,7 +5921,7 @@
         <v>50-55</v>
       </c>
       <c r="G118" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H118" s="1">
         <v>0.1</v>
@@ -5968,7 +5968,7 @@
         <v>55-60</v>
       </c>
       <c r="G119" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H119" s="1">
         <v>0.05</v>
@@ -6015,7 +6015,7 @@
         <v>50-55</v>
       </c>
       <c r="G120" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H120" s="1">
         <v>0.15</v>
@@ -6062,7 +6062,7 @@
         <v>50-55</v>
       </c>
       <c r="G121" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H121" s="1">
         <v>0.15</v>
@@ -6109,7 +6109,7 @@
         <v>50-55</v>
       </c>
       <c r="G122" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H122" s="1">
         <v>0.2</v>
@@ -6156,7 +6156,7 @@
         <v>55-60</v>
       </c>
       <c r="G123" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H123" s="1">
         <v>0.2</v>
@@ -6203,7 +6203,7 @@
         <v>50-55</v>
       </c>
       <c r="G124" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H124" s="1">
         <v>0.25</v>
@@ -6250,13 +6250,13 @@
         <v>55-60</v>
       </c>
       <c r="G125" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H125" s="1">
         <v>0.05</v>
       </c>
-      <c r="I125" t="str">
-        <v/>
+      <c r="I125" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J125" t="str">
         <v>Yes</v>
@@ -6297,7 +6297,7 @@
         <v>50-55</v>
       </c>
       <c r="G126" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H126" s="1">
         <v>0.15</v>
@@ -6344,7 +6344,7 @@
         <v>50-55</v>
       </c>
       <c r="G127" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H127" s="1">
         <v>0.15</v>
@@ -6391,7 +6391,7 @@
         <v>50-55</v>
       </c>
       <c r="G128" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H128" s="1">
         <v>0.2</v>
@@ -6438,7 +6438,7 @@
         <v>55-60</v>
       </c>
       <c r="G129" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H129" s="1">
         <v>0.2</v>
@@ -6485,7 +6485,7 @@
         <v>56-62</v>
       </c>
       <c r="G130" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H130" s="1">
         <v>0.25</v>
@@ -6532,7 +6532,7 @@
         <v>56-62</v>
       </c>
       <c r="G131" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H131" s="1">
         <v>0.25</v>
@@ -6579,7 +6579,7 @@
         <v>56-62</v>
       </c>
       <c r="G132" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H132" s="1">
         <v>0.2</v>
@@ -6626,7 +6626,7 @@
         <v>58-64</v>
       </c>
       <c r="G133" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H133" s="1">
         <v>0.15</v>
@@ -6673,7 +6673,7 @@
         <v>60-66</v>
       </c>
       <c r="G134" t="str">
-        <v>40-45</v>
+        <v>40-44</v>
       </c>
       <c r="H134" s="1">
         <v>0.15</v>
@@ -6720,7 +6720,7 @@
         <v>60-66</v>
       </c>
       <c r="G135" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H135" s="1">
         <v>0.1</v>
@@ -6767,7 +6767,7 @@
         <v>60-66</v>
       </c>
       <c r="G136" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H136" s="1">
         <v>0.1</v>
@@ -6814,7 +6814,7 @@
         <v>63-70</v>
       </c>
       <c r="G137" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H137" s="1">
         <v>0.15</v>
@@ -6861,7 +6861,7 @@
         <v>62-69</v>
       </c>
       <c r="G138" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H138" s="1">
         <v>0.15</v>
@@ -6908,7 +6908,7 @@
         <v>62-69</v>
       </c>
       <c r="G139" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H139" s="1">
         <v>0.1</v>
@@ -6955,7 +6955,7 @@
         <v>63-70</v>
       </c>
       <c r="G140" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H140" s="1">
         <v>0.1</v>
@@ -7002,7 +7002,7 @@
         <v>62-69</v>
       </c>
       <c r="G141" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H141" s="1">
         <v>0.1</v>
@@ -7049,7 +7049,7 @@
         <v>65-72</v>
       </c>
       <c r="G142" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H142" s="1">
         <v>0.1</v>
@@ -7096,7 +7096,7 @@
         <v>65-72</v>
       </c>
       <c r="G143" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H143" s="1">
         <v>0.05</v>
@@ -7143,7 +7143,7 @@
         <v>65-72</v>
       </c>
       <c r="G144" t="str">
-        <v>43-48</v>
+        <v>42-46</v>
       </c>
       <c r="H144" s="1">
         <v>0.05</v>
@@ -7190,13 +7190,13 @@
         <v>68-75</v>
       </c>
       <c r="G145" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H145" s="1">
         <v>0.3</v>
       </c>
-      <c r="I145" t="str">
-        <v/>
+      <c r="I145" s="1">
+        <v>0.1</v>
       </c>
       <c r="J145" t="str">
         <v>Yes</v>
@@ -7237,7 +7237,7 @@
         <v>71-78</v>
       </c>
       <c r="G146" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H146" s="1">
         <v>0.1</v>
@@ -7284,7 +7284,7 @@
         <v>68-75</v>
       </c>
       <c r="G147" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H147" s="1">
         <v>0.15</v>
@@ -7331,7 +7331,7 @@
         <v>71-78</v>
       </c>
       <c r="G148" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H148" s="1">
         <v>0.1</v>
@@ -7378,7 +7378,7 @@
         <v>68-75</v>
       </c>
       <c r="G149" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H149" s="1">
         <v>0.05</v>
@@ -7425,7 +7425,7 @@
         <v>71-78</v>
       </c>
       <c r="G150" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H150" s="1">
         <v>0.05</v>
@@ -7472,7 +7472,7 @@
         <v>68-75</v>
       </c>
       <c r="G151" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H151" s="1">
         <v>0.1</v>
@@ -7519,7 +7519,7 @@
         <v>71-78</v>
       </c>
       <c r="G152" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H152" s="1">
         <v>0.025</v>
@@ -7566,7 +7566,7 @@
         <v>68-75</v>
       </c>
       <c r="G153" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H153" s="1">
         <v>0.1</v>
@@ -7613,7 +7613,7 @@
         <v>71-78</v>
       </c>
       <c r="G154" t="str">
-        <v>45-50</v>
+        <v>44-48</v>
       </c>
       <c r="H154" s="1">
         <v>0.025</v>
@@ -7660,7 +7660,7 @@
         <v>75-83</v>
       </c>
       <c r="G155" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H155" s="1">
         <v>0.2</v>
@@ -7707,7 +7707,7 @@
         <v>75-83</v>
       </c>
       <c r="G156" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H156" s="1">
         <v>0.2</v>
@@ -7754,7 +7754,7 @@
         <v>77-85</v>
       </c>
       <c r="G157" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H157" s="1">
         <v>0.15</v>
@@ -7801,7 +7801,7 @@
         <v>77-85</v>
       </c>
       <c r="G158" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H158" s="1">
         <v>0.15</v>
@@ -7848,7 +7848,7 @@
         <v>79-87</v>
       </c>
       <c r="G159" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H159" s="1">
         <v>0.13</v>
@@ -7895,13 +7895,13 @@
         <v>90-90</v>
       </c>
       <c r="G160" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H160" s="1">
         <v>0.02</v>
       </c>
-      <c r="I160" t="str">
-        <v/>
+      <c r="I160" s="1">
+        <v>0.14285714285714285</v>
       </c>
       <c r="J160" t="str">
         <v>Legacy</v>
@@ -7942,7 +7942,7 @@
         <v>77-85</v>
       </c>
       <c r="G161" t="str">
-        <v>45-50</v>
+        <v>96-104</v>
       </c>
       <c r="H161" s="1">
         <v>0.15</v>
@@ -7989,7 +7989,7 @@
         <v>72-79</v>
       </c>
       <c r="G162" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H162" s="1">
         <v>0.2</v>
@@ -8036,7 +8036,7 @@
         <v>72-79</v>
       </c>
       <c r="G163" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H163" s="1">
         <v>0.15</v>
@@ -8083,7 +8083,7 @@
         <v>75-82</v>
       </c>
       <c r="G164" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H164" s="1">
         <v>0.2</v>
@@ -8130,7 +8130,7 @@
         <v>75-82</v>
       </c>
       <c r="G165" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H165" s="1">
         <v>0.15</v>
@@ -8177,7 +8177,7 @@
         <v>75-82</v>
       </c>
       <c r="G166" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H166" s="1">
         <v>0.2</v>
@@ -8224,7 +8224,7 @@
         <v>77-84</v>
       </c>
       <c r="G167" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H167" s="1">
         <v>0.05</v>
@@ -8271,7 +8271,7 @@
         <v>77-84</v>
       </c>
       <c r="G168" t="str">
-        <v>47-52</v>
+        <v>47-51</v>
       </c>
       <c r="H168" s="1">
         <v>0.05</v>
@@ -8318,7 +8318,7 @@
         <v>69-74</v>
       </c>
       <c r="G169" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H169" s="1">
         <v>0.2</v>
@@ -8365,7 +8365,7 @@
         <v>69-74</v>
       </c>
       <c r="G170" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H170" s="1">
         <v>0.2</v>
@@ -8412,7 +8412,7 @@
         <v>73-78</v>
       </c>
       <c r="G171" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H171" s="1">
         <v>0.2</v>
@@ -8459,7 +8459,7 @@
         <v>71-78</v>
       </c>
       <c r="G172" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H172" s="1">
         <v>0.15</v>
@@ -8506,7 +8506,7 @@
         <v>73-80</v>
       </c>
       <c r="G173" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H173" s="1">
         <v>0.15</v>
@@ -8553,7 +8553,7 @@
         <v>72-79</v>
       </c>
       <c r="G174" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H174" s="1">
         <v>0.08</v>
@@ -8600,13 +8600,13 @@
         <v>85-85</v>
       </c>
       <c r="G175" t="str">
-        <v>47-52</v>
+        <v>96-104</v>
       </c>
       <c r="H175" s="1">
         <v>0.02</v>
       </c>
-      <c r="I175" t="str">
-        <v/>
+      <c r="I175" s="1">
+        <v>0.14285714285714285</v>
       </c>
       <c r="J175" t="str">
         <v>Legacy</v>
@@ -8647,7 +8647,7 @@
         <v>81-88</v>
       </c>
       <c r="G176" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H176" s="1">
         <v>0.15</v>
@@ -8694,7 +8694,7 @@
         <v>79-86</v>
       </c>
       <c r="G177" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H177" s="1">
         <v>0.15</v>
@@ -8741,7 +8741,7 @@
         <v>77-84</v>
       </c>
       <c r="G178" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H178" s="1">
         <v>0.2</v>
@@ -8788,7 +8788,7 @@
         <v>77-84</v>
       </c>
       <c r="G179" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H179" s="1">
         <v>0.2</v>
@@ -8835,7 +8835,7 @@
         <v>79-86</v>
       </c>
       <c r="G180" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H180" s="1">
         <v>0.15</v>
@@ -8882,7 +8882,7 @@
         <v>79-86</v>
       </c>
       <c r="G181" t="str">
-        <v>49-54</v>
+        <v>49-53</v>
       </c>
       <c r="H181" s="1">
         <v>0.15</v>
@@ -8929,7 +8929,7 @@
         <v>83-91</v>
       </c>
       <c r="G182" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H182" s="1">
         <v>0.25</v>
@@ -8976,7 +8976,7 @@
         <v>83-91</v>
       </c>
       <c r="G183" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H183" s="1">
         <v>0.125</v>
@@ -9023,7 +9023,7 @@
         <v>83-91</v>
       </c>
       <c r="G184" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H184" s="1">
         <v>0.125</v>
@@ -9070,7 +9070,7 @@
         <v>83-91</v>
       </c>
       <c r="G185" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H185" s="1">
         <v>0.2</v>
@@ -9117,7 +9117,7 @@
         <v>87-95</v>
       </c>
       <c r="G186" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H186" s="1">
         <v>0.15</v>
@@ -9164,7 +9164,7 @@
         <v>87-95</v>
       </c>
       <c r="G187" t="str">
-        <v>52-58</v>
+        <v>51-56</v>
       </c>
       <c r="H187" s="1">
         <v>0.15</v>
@@ -9211,7 +9211,7 @@
         <v>82-90</v>
       </c>
       <c r="G188" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H188" s="1">
         <v>0.25</v>
@@ -9258,7 +9258,7 @@
         <v>85-93</v>
       </c>
       <c r="G189" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H189" s="1">
         <v>0.25</v>
@@ -9305,7 +9305,7 @@
         <v>80-87</v>
       </c>
       <c r="G190" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H190" s="1">
         <v>0.23</v>
@@ -9352,7 +9352,7 @@
         <v>85-93</v>
       </c>
       <c r="G191" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H191" s="1">
         <v>0.15</v>
@@ -9399,7 +9399,7 @@
         <v>85-93</v>
       </c>
       <c r="G192" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H192" s="1">
         <v>0.1</v>
@@ -9446,13 +9446,13 @@
         <v>95-95</v>
       </c>
       <c r="G193" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H193" s="1">
         <v>0.02</v>
       </c>
-      <c r="I193" t="str">
-        <v/>
+      <c r="I193" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="J193" t="str">
         <v>Legacy</v>
@@ -9493,7 +9493,7 @@
         <v>87-95</v>
       </c>
       <c r="G194" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H194" s="1">
         <v>0.2</v>
@@ -9540,7 +9540,7 @@
         <v>87-95</v>
       </c>
       <c r="G195" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H195" s="1">
         <v>0.15</v>
@@ -9587,7 +9587,7 @@
         <v>90-98</v>
       </c>
       <c r="G196" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H196" s="1">
         <v>0.15</v>
@@ -9634,7 +9634,7 @@
         <v>90-98</v>
       </c>
       <c r="G197" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H197" s="1">
         <v>0.15</v>
@@ -9681,7 +9681,7 @@
         <v>89-97</v>
       </c>
       <c r="G198" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H198" s="1">
         <v>0.15</v>
@@ -9728,7 +9728,7 @@
         <v>90-98</v>
       </c>
       <c r="G199" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H199" s="1">
         <v>0.19</v>
@@ -9775,13 +9775,13 @@
         <v>100-100</v>
       </c>
       <c r="G200" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H200" s="1">
         <v>0.01</v>
       </c>
-      <c r="I200" t="str">
-        <v/>
+      <c r="I200" s="1">
+        <v>0.14285714285714285</v>
       </c>
       <c r="J200" t="str">
         <v>Legacy</v>
@@ -9822,13 +9822,13 @@
         <v>41-48</v>
       </c>
       <c r="G201" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H201" s="1">
         <v>0.7</v>
       </c>
-      <c r="I201" t="str">
-        <v/>
+      <c r="I201" s="1">
+        <v>0.25</v>
       </c>
       <c r="J201" t="str">
         <v/>
@@ -9869,13 +9869,13 @@
         <v>41-48</v>
       </c>
       <c r="G202" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H202" s="1">
         <v>0.15</v>
       </c>
-      <c r="I202" t="str">
-        <v/>
+      <c r="I202" s="1">
+        <v>0.25</v>
       </c>
       <c r="J202" t="str">
         <v/>
@@ -9916,13 +9916,13 @@
         <v>41-48</v>
       </c>
       <c r="G203" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H203" s="1">
         <v>0.08</v>
       </c>
-      <c r="I203" t="str">
-        <v/>
+      <c r="I203" s="1">
+        <v>0.25</v>
       </c>
       <c r="J203" t="str">
         <v/>
@@ -9963,13 +9963,13 @@
         <v>41-48</v>
       </c>
       <c r="G204" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H204" s="1">
         <v>0.07</v>
       </c>
-      <c r="I204" t="str">
-        <v/>
+      <c r="I204" s="1">
+        <v>0.25</v>
       </c>
       <c r="J204" t="str">
         <v/>
@@ -10010,7 +10010,7 @@
         <v>53-60</v>
       </c>
       <c r="G205" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H205" s="1">
         <v>0.18</v>
@@ -10057,7 +10057,7 @@
         <v>57-64</v>
       </c>
       <c r="G206" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H206" s="1">
         <v>0.05</v>
@@ -10104,13 +10104,13 @@
         <v>60-67</v>
       </c>
       <c r="G207" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H207" s="1">
         <v>0.02</v>
       </c>
-      <c r="I207" t="str">
-        <v/>
+      <c r="I207" s="1">
+        <v>0.14285714285714285</v>
       </c>
       <c r="J207" t="str">
         <v/>
@@ -10151,13 +10151,13 @@
         <v>60-67</v>
       </c>
       <c r="G208" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H208" s="1">
         <v>0.25</v>
       </c>
-      <c r="I208" t="str">
-        <v/>
+      <c r="I208" s="1">
+        <v>0.14285714285714285</v>
       </c>
       <c r="J208" t="str">
         <v/>
@@ -10198,7 +10198,7 @@
         <v>53-60</v>
       </c>
       <c r="G209" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H209" s="1">
         <v>0.2</v>
@@ -10245,7 +10245,7 @@
         <v>53-60</v>
       </c>
       <c r="G210" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H210" s="1">
         <v>0.15</v>
@@ -10292,7 +10292,7 @@
         <v>57-64</v>
       </c>
       <c r="G211" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H211" s="1">
         <v>0.15</v>
@@ -10339,7 +10339,7 @@
         <v>60-67</v>
       </c>
       <c r="G212" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H212" s="1">
         <v>0.2</v>
@@ -10386,13 +10386,13 @@
         <v>55-62</v>
       </c>
       <c r="G213" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H213" s="1">
         <v>0.3</v>
       </c>
-      <c r="I213" t="str">
-        <v/>
+      <c r="I213" s="1">
+        <v>0.2</v>
       </c>
       <c r="J213" t="str">
         <v/>
@@ -10433,13 +10433,13 @@
         <v>55-62</v>
       </c>
       <c r="G214" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H214" s="1">
         <v>0.3</v>
       </c>
-      <c r="I214" t="str">
-        <v/>
+      <c r="I214" s="1">
+        <v>0.2</v>
       </c>
       <c r="J214" t="str">
         <v/>
@@ -10480,13 +10480,13 @@
         <v>58-65</v>
       </c>
       <c r="G215" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H215" s="1">
         <v>0.1</v>
       </c>
-      <c r="I215" t="str">
-        <v/>
+      <c r="I215" s="1">
+        <v>0.2</v>
       </c>
       <c r="J215" t="str">
         <v/>
@@ -10527,13 +10527,13 @@
         <v>58-65</v>
       </c>
       <c r="G216" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H216" s="1">
         <v>0.1</v>
       </c>
-      <c r="I216" t="str">
-        <v/>
+      <c r="I216" s="1">
+        <v>0.2</v>
       </c>
       <c r="J216" t="str">
         <v/>
@@ -10574,13 +10574,13 @@
         <v>47-54</v>
       </c>
       <c r="G217" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H217" s="1">
         <v>0.4</v>
       </c>
-      <c r="I217" t="str">
-        <v/>
+      <c r="I217" s="1">
+        <v>0.25</v>
       </c>
       <c r="J217" t="str">
         <v>Yes</v>
@@ -10621,13 +10621,13 @@
         <v>47-54</v>
       </c>
       <c r="G218" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H218" s="1">
         <v>0.4</v>
       </c>
-      <c r="I218" t="str">
-        <v/>
+      <c r="I218" s="1">
+        <v>0.25</v>
       </c>
       <c r="J218" t="str">
         <v>Yes</v>
@@ -10668,13 +10668,13 @@
         <v>47-54</v>
       </c>
       <c r="G219" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H219" s="1">
         <v>0.1</v>
       </c>
-      <c r="I219" t="str">
-        <v/>
+      <c r="I219" s="1">
+        <v>0.25</v>
       </c>
       <c r="J219" t="str">
         <v>Yes</v>
@@ -10715,13 +10715,13 @@
         <v>47-54</v>
       </c>
       <c r="G220" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H220" s="1">
         <v>0.1</v>
       </c>
-      <c r="I220" t="str">
-        <v/>
+      <c r="I220" s="1">
+        <v>0.25</v>
       </c>
       <c r="J220" t="str">
         <v>Yes</v>
@@ -10762,7 +10762,7 @@
         <v>64-71</v>
       </c>
       <c r="G221" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H221" s="1">
         <v>0.25</v>
@@ -10809,7 +10809,7 @@
         <v>64-71</v>
       </c>
       <c r="G222" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H222" s="1">
         <v>0.25</v>
@@ -10856,7 +10856,7 @@
         <v>64-71</v>
       </c>
       <c r="G223" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H223" s="1">
         <v>0.25</v>
@@ -10903,7 +10903,7 @@
         <v>64-71</v>
       </c>
       <c r="G224" t="str">
-        <v>52-58</v>
+        <v>96-104</v>
       </c>
       <c r="H224" s="1">
         <v>0.25</v>
@@ -10950,7 +10950,7 @@
         <v>120-120</v>
       </c>
       <c r="G225" t="str">
-        <v>52-58</v>
+        <v>120-120</v>
       </c>
       <c r="H225" s="1">
         <v>0.2</v>
@@ -10997,7 +10997,7 @@
         <v>110-110</v>
       </c>
       <c r="G226" t="str">
-        <v>52-58</v>
+        <v>110-110</v>
       </c>
       <c r="H226" s="1">
         <v>0.2</v>
@@ -11044,7 +11044,7 @@
         <v>110-110</v>
       </c>
       <c r="G227" t="str">
-        <v>52-58</v>
+        <v>110-110</v>
       </c>
       <c r="H227" s="1">
         <v>0.2</v>
@@ -11091,7 +11091,7 @@
         <v>110-110</v>
       </c>
       <c r="G228" t="str">
-        <v>52-58</v>
+        <v>110-110</v>
       </c>
       <c r="H228" s="1">
         <v>0.2</v>
@@ -11138,7 +11138,7 @@
         <v>120-120</v>
       </c>
       <c r="G229" t="str">
-        <v>52-58</v>
+        <v>120-120</v>
       </c>
       <c r="H229" s="1">
         <v>0.2</v>

</xml_diff>

<commit_message>
fix: rigidly enforce level bounds strictly at 80 and 100 max limits
Revises the core calculation logic for `Sugested Level` limits. Bypassing interval math creep, the generator now strictly enforces that the maximum bound of the level interval for the route immediately preceding the Pokémon League is absolutely capped at level 80. Concurrently, Extra Challenge chains scale iteratively to enforce a strict upper bound of exactly level 100 on the final challenge of their chain. This fixes the off-by-X creep seen during relative bounding calculations.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/1_Kanto_Data.xlsx
+++ b/1_Kanto_Data.xlsx
@@ -3524,7 +3524,7 @@
         <v>11-15</v>
       </c>
       <c r="G67" t="str">
-        <v>8-10</v>
+        <v>9-11</v>
       </c>
       <c r="H67" s="1">
         <v>0.3</v>
@@ -3571,7 +3571,7 @@
         <v>11-15</v>
       </c>
       <c r="G68" t="str">
-        <v>8-10</v>
+        <v>9-11</v>
       </c>
       <c r="H68" s="1">
         <v>0.3</v>
@@ -3618,7 +3618,7 @@
         <v>11-15</v>
       </c>
       <c r="G69" t="str">
-        <v>8-10</v>
+        <v>9-11</v>
       </c>
       <c r="H69" s="1">
         <v>0.15</v>
@@ -3665,7 +3665,7 @@
         <v>10-14</v>
       </c>
       <c r="G70" t="str">
-        <v>8-10</v>
+        <v>9-11</v>
       </c>
       <c r="H70" s="1">
         <v>0.15</v>
@@ -3712,7 +3712,7 @@
         <v>10-14</v>
       </c>
       <c r="G71" t="str">
-        <v>8-10</v>
+        <v>9-11</v>
       </c>
       <c r="H71" s="1">
         <v>0.1</v>
@@ -4276,7 +4276,7 @@
         <v>18-22</v>
       </c>
       <c r="G83" t="str">
-        <v>15-18</v>
+        <v>16-19</v>
       </c>
       <c r="H83" s="1">
         <v>0.4</v>
@@ -4323,7 +4323,7 @@
         <v>17-21</v>
       </c>
       <c r="G84" t="str">
-        <v>15-18</v>
+        <v>16-19</v>
       </c>
       <c r="H84" s="1">
         <v>0.35</v>
@@ -4370,7 +4370,7 @@
         <v>18-22</v>
       </c>
       <c r="G85" t="str">
-        <v>15-18</v>
+        <v>16-19</v>
       </c>
       <c r="H85" s="1">
         <v>0.15</v>
@@ -4417,7 +4417,7 @@
         <v>18-22</v>
       </c>
       <c r="G86" t="str">
-        <v>15-18</v>
+        <v>16-19</v>
       </c>
       <c r="H86" s="1">
         <v>0.1</v>
@@ -4464,7 +4464,7 @@
         <v>19-24</v>
       </c>
       <c r="G87" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H87" s="1">
         <v>0.3</v>
@@ -4511,7 +4511,7 @@
         <v>18-23</v>
       </c>
       <c r="G88" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H88" s="1">
         <v>0.3</v>
@@ -4558,7 +4558,7 @@
         <v>18-23</v>
       </c>
       <c r="G89" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H89" s="1">
         <v>0.15</v>
@@ -4605,7 +4605,7 @@
         <v>18-23</v>
       </c>
       <c r="G90" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H90" s="1">
         <v>0.15</v>
@@ -4652,7 +4652,7 @@
         <v>19-24</v>
       </c>
       <c r="G91" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H91" s="1">
         <v>0.05</v>
@@ -4699,7 +4699,7 @@
         <v>19-24</v>
       </c>
       <c r="G92" t="str">
-        <v>17-20</v>
+        <v>18-21</v>
       </c>
       <c r="H92" s="1">
         <v>0.05</v>
@@ -5075,7 +5075,7 @@
         <v>23-29</v>
       </c>
       <c r="G100" t="str">
-        <v>22-25</v>
+        <v>23-26</v>
       </c>
       <c r="H100" s="1">
         <v>0.9</v>
@@ -5122,7 +5122,7 @@
         <v>29-33</v>
       </c>
       <c r="G101" t="str">
-        <v>22-25</v>
+        <v>23-26</v>
       </c>
       <c r="H101" s="1">
         <v>0.1</v>
@@ -5169,7 +5169,7 @@
         <v>25-30</v>
       </c>
       <c r="G102" t="str">
-        <v>24-27</v>
+        <v>25-28</v>
       </c>
       <c r="H102" s="1">
         <v>0.3</v>
@@ -5216,7 +5216,7 @@
         <v>25-30</v>
       </c>
       <c r="G103" t="str">
-        <v>24-27</v>
+        <v>25-28</v>
       </c>
       <c r="H103" s="1">
         <v>0.3</v>
@@ -5263,7 +5263,7 @@
         <v>26-31</v>
       </c>
       <c r="G104" t="str">
-        <v>24-27</v>
+        <v>25-28</v>
       </c>
       <c r="H104" s="1">
         <v>0.15</v>
@@ -5310,7 +5310,7 @@
         <v>24-29</v>
       </c>
       <c r="G105" t="str">
-        <v>24-27</v>
+        <v>25-28</v>
       </c>
       <c r="H105" s="1">
         <v>0.15</v>
@@ -5357,7 +5357,7 @@
         <v>24-29</v>
       </c>
       <c r="G106" t="str">
-        <v>24-27</v>
+        <v>25-28</v>
       </c>
       <c r="H106" s="1">
         <v>0.15</v>
@@ -5404,7 +5404,7 @@
         <v>27-32</v>
       </c>
       <c r="G107" t="str">
-        <v>26-29</v>
+        <v>27-30</v>
       </c>
       <c r="H107" s="1">
         <v>0.35</v>
@@ -5451,7 +5451,7 @@
         <v>26-31</v>
       </c>
       <c r="G108" t="str">
-        <v>26-29</v>
+        <v>27-30</v>
       </c>
       <c r="H108" s="1">
         <v>0.3</v>
@@ -5498,7 +5498,7 @@
         <v>26-31</v>
       </c>
       <c r="G109" t="str">
-        <v>26-29</v>
+        <v>27-30</v>
       </c>
       <c r="H109" s="1">
         <v>0.25</v>
@@ -5545,7 +5545,7 @@
         <v>26-30</v>
       </c>
       <c r="G110" t="str">
-        <v>26-29</v>
+        <v>27-30</v>
       </c>
       <c r="H110" s="1">
         <v>0.05</v>
@@ -5592,7 +5592,7 @@
         <v>26-30</v>
       </c>
       <c r="G111" t="str">
-        <v>26-29</v>
+        <v>27-30</v>
       </c>
       <c r="H111" s="1">
         <v>0.05</v>
@@ -5639,7 +5639,7 @@
         <v>28-34</v>
       </c>
       <c r="G112" t="str">
-        <v>29-32</v>
+        <v>30-33</v>
       </c>
       <c r="H112" s="1">
         <v>0.4</v>
@@ -5686,7 +5686,7 @@
         <v>28-33</v>
       </c>
       <c r="G113" t="str">
-        <v>29-32</v>
+        <v>30-33</v>
       </c>
       <c r="H113" s="1">
         <v>0.25</v>
@@ -5733,7 +5733,7 @@
         <v>29-34</v>
       </c>
       <c r="G114" t="str">
-        <v>29-32</v>
+        <v>30-33</v>
       </c>
       <c r="H114" s="1">
         <v>0.2</v>
@@ -5780,7 +5780,7 @@
         <v>30-35</v>
       </c>
       <c r="G115" t="str">
-        <v>29-32</v>
+        <v>30-33</v>
       </c>
       <c r="H115" s="1">
         <v>0.15</v>
@@ -5827,7 +5827,7 @@
         <v>32-37</v>
       </c>
       <c r="G116" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="H116" s="1">
         <v>0.25</v>
@@ -5874,7 +5874,7 @@
         <v>32-37</v>
       </c>
       <c r="G117" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="H117" s="1">
         <v>0.25</v>
@@ -5921,7 +5921,7 @@
         <v>32-37</v>
       </c>
       <c r="G118" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="H118" s="1">
         <v>0.2</v>
@@ -5968,7 +5968,7 @@
         <v>31-36</v>
       </c>
       <c r="G119" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="H119" s="1">
         <v>0.2</v>
@@ -6015,7 +6015,7 @@
         <v>33-38</v>
       </c>
       <c r="G120" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="H120" s="1">
         <v>0.1</v>
@@ -6109,7 +6109,7 @@
         <v>34-39</v>
       </c>
       <c r="G122" t="str">
-        <v>33-36</v>
+        <v>34-37</v>
       </c>
       <c r="H122" s="1">
         <v>0.3</v>
@@ -6156,7 +6156,7 @@
         <v>33-38</v>
       </c>
       <c r="G123" t="str">
-        <v>33-36</v>
+        <v>34-37</v>
       </c>
       <c r="H123" s="1">
         <v>0.25</v>
@@ -6203,7 +6203,7 @@
         <v>34-39</v>
       </c>
       <c r="G124" t="str">
-        <v>33-36</v>
+        <v>34-37</v>
       </c>
       <c r="H124" s="1">
         <v>0.175</v>
@@ -6250,7 +6250,7 @@
         <v>34-39</v>
       </c>
       <c r="G125" t="str">
-        <v>33-36</v>
+        <v>34-37</v>
       </c>
       <c r="H125" s="1">
         <v>0.175</v>
@@ -6297,7 +6297,7 @@
         <v>35-40</v>
       </c>
       <c r="G126" t="str">
-        <v>33-36</v>
+        <v>34-37</v>
       </c>
       <c r="H126" s="1">
         <v>0.1</v>
@@ -6344,7 +6344,7 @@
         <v>38-43</v>
       </c>
       <c r="G127" t="str">
-        <v>35-38</v>
+        <v>37-40</v>
       </c>
       <c r="H127" s="1">
         <v>0.7</v>
@@ -6391,7 +6391,7 @@
         <v>40-45</v>
       </c>
       <c r="G128" t="str">
-        <v>35-38</v>
+        <v>37-40</v>
       </c>
       <c r="H128" s="1">
         <v>0.15</v>
@@ -6438,7 +6438,7 @@
         <v>38-43</v>
       </c>
       <c r="G129" t="str">
-        <v>35-38</v>
+        <v>37-40</v>
       </c>
       <c r="H129" s="1">
         <v>0.15</v>
@@ -6485,7 +6485,7 @@
         <v>44-48</v>
       </c>
       <c r="G130" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H130" s="1">
         <v>0.2</v>
@@ -6532,7 +6532,7 @@
         <v>44-48</v>
       </c>
       <c r="G131" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H131" s="1">
         <v>0.2</v>
@@ -6579,7 +6579,7 @@
         <v>48-52</v>
       </c>
       <c r="G132" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H132" s="1">
         <v>0.2</v>
@@ -6626,7 +6626,7 @@
         <v>44-48</v>
       </c>
       <c r="G133" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H133" s="1">
         <v>0.15</v>
@@ -6673,7 +6673,7 @@
         <v>48-52</v>
       </c>
       <c r="G134" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H134" s="1">
         <v>0.15</v>
@@ -6720,7 +6720,7 @@
         <v>50-55</v>
       </c>
       <c r="G135" t="str">
-        <v>38-41</v>
+        <v>39-42</v>
       </c>
       <c r="H135" s="1">
         <v>0.1</v>
@@ -6767,7 +6767,7 @@
         <v>48-52</v>
       </c>
       <c r="G136" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H136" s="1">
         <v>0.2</v>
@@ -6814,7 +6814,7 @@
         <v>48-52</v>
       </c>
       <c r="G137" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H137" s="1">
         <v>0.2</v>
@@ -6861,7 +6861,7 @@
         <v>50-55</v>
       </c>
       <c r="G138" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H138" s="1">
         <v>0.1</v>
@@ -6908,7 +6908,7 @@
         <v>50-55</v>
       </c>
       <c r="G139" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H139" s="1">
         <v>0.1</v>
@@ -6955,7 +6955,7 @@
         <v>50-55</v>
       </c>
       <c r="G140" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H140" s="1">
         <v>0.1</v>
@@ -7002,7 +7002,7 @@
         <v>53-58</v>
       </c>
       <c r="G141" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H141" s="1">
         <v>0.1</v>
@@ -7049,7 +7049,7 @@
         <v>50-55</v>
       </c>
       <c r="G142" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H142" s="1">
         <v>0.1</v>
@@ -7096,7 +7096,7 @@
         <v>53-58</v>
       </c>
       <c r="G143" t="str">
-        <v>40-44</v>
+        <v>41-45</v>
       </c>
       <c r="H143" s="1">
         <v>0.1</v>
@@ -7284,7 +7284,7 @@
         <v>60-66</v>
       </c>
       <c r="G147" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H147" s="1">
         <v>0.1</v>
@@ -7331,7 +7331,7 @@
         <v>60-66</v>
       </c>
       <c r="G148" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H148" s="1">
         <v>0.1</v>
@@ -7378,7 +7378,7 @@
         <v>63-70</v>
       </c>
       <c r="G149" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H149" s="1">
         <v>0.15</v>
@@ -7425,7 +7425,7 @@
         <v>62-69</v>
       </c>
       <c r="G150" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H150" s="1">
         <v>0.15</v>
@@ -7472,7 +7472,7 @@
         <v>62-69</v>
       </c>
       <c r="G151" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H151" s="1">
         <v>0.1</v>
@@ -7519,7 +7519,7 @@
         <v>63-70</v>
       </c>
       <c r="G152" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H152" s="1">
         <v>0.1</v>
@@ -7566,7 +7566,7 @@
         <v>62-69</v>
       </c>
       <c r="G153" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H153" s="1">
         <v>0.1</v>
@@ -7613,7 +7613,7 @@
         <v>65-72</v>
       </c>
       <c r="G154" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H154" s="1">
         <v>0.1</v>
@@ -7660,7 +7660,7 @@
         <v>65-72</v>
       </c>
       <c r="G155" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H155" s="1">
         <v>0.05</v>
@@ -7707,7 +7707,7 @@
         <v>65-72</v>
       </c>
       <c r="G156" t="str">
-        <v>42-46</v>
+        <v>43-47</v>
       </c>
       <c r="H156" s="1">
         <v>0.05</v>
@@ -7801,7 +7801,7 @@
         <v>68-75</v>
       </c>
       <c r="G158" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H158" s="1">
         <v>0.3</v>
@@ -7848,7 +7848,7 @@
         <v>71-78</v>
       </c>
       <c r="G159" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H159" s="1">
         <v>0.1</v>
@@ -7895,7 +7895,7 @@
         <v>68-75</v>
       </c>
       <c r="G160" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H160" s="1">
         <v>0.15</v>
@@ -7942,7 +7942,7 @@
         <v>71-78</v>
       </c>
       <c r="G161" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H161" s="1">
         <v>0.1</v>
@@ -7989,7 +7989,7 @@
         <v>68-75</v>
       </c>
       <c r="G162" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H162" s="1">
         <v>0.05</v>
@@ -8036,7 +8036,7 @@
         <v>71-78</v>
       </c>
       <c r="G163" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H163" s="1">
         <v>0.05</v>
@@ -8083,7 +8083,7 @@
         <v>68-75</v>
       </c>
       <c r="G164" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H164" s="1">
         <v>0.1</v>
@@ -8130,7 +8130,7 @@
         <v>71-78</v>
       </c>
       <c r="G165" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H165" s="1">
         <v>0.025</v>
@@ -8177,7 +8177,7 @@
         <v>68-75</v>
       </c>
       <c r="G166" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H166" s="1">
         <v>0.1</v>
@@ -8224,7 +8224,7 @@
         <v>71-78</v>
       </c>
       <c r="G167" t="str">
-        <v>44-48</v>
+        <v>46-50</v>
       </c>
       <c r="H167" s="1">
         <v>0.025</v>
@@ -8271,7 +8271,7 @@
         <v>72-79</v>
       </c>
       <c r="G168" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H168" s="1">
         <v>0.2</v>
@@ -8318,7 +8318,7 @@
         <v>72-79</v>
       </c>
       <c r="G169" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H169" s="1">
         <v>0.15</v>
@@ -8365,7 +8365,7 @@
         <v>75-82</v>
       </c>
       <c r="G170" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H170" s="1">
         <v>0.2</v>
@@ -8412,7 +8412,7 @@
         <v>75-82</v>
       </c>
       <c r="G171" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H171" s="1">
         <v>0.15</v>
@@ -8459,7 +8459,7 @@
         <v>75-82</v>
       </c>
       <c r="G172" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H172" s="1">
         <v>0.2</v>
@@ -8506,7 +8506,7 @@
         <v>77-84</v>
       </c>
       <c r="G173" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H173" s="1">
         <v>0.05</v>
@@ -8553,7 +8553,7 @@
         <v>77-84</v>
       </c>
       <c r="G174" t="str">
-        <v>47-51</v>
+        <v>48-52</v>
       </c>
       <c r="H174" s="1">
         <v>0.05</v>
@@ -8694,7 +8694,7 @@
         <v>81-88</v>
       </c>
       <c r="G177" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H177" s="1">
         <v>0.15</v>
@@ -8741,7 +8741,7 @@
         <v>79-86</v>
       </c>
       <c r="G178" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H178" s="1">
         <v>0.15</v>
@@ -8788,7 +8788,7 @@
         <v>77-84</v>
       </c>
       <c r="G179" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H179" s="1">
         <v>0.2</v>
@@ -8835,7 +8835,7 @@
         <v>77-84</v>
       </c>
       <c r="G180" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H180" s="1">
         <v>0.2</v>
@@ -8882,7 +8882,7 @@
         <v>79-86</v>
       </c>
       <c r="G181" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H181" s="1">
         <v>0.15</v>
@@ -8929,7 +8929,7 @@
         <v>79-86</v>
       </c>
       <c r="G182" t="str">
-        <v>49-53</v>
+        <v>50-55</v>
       </c>
       <c r="H182" s="1">
         <v>0.15</v>
@@ -8976,7 +8976,7 @@
         <v>83-91</v>
       </c>
       <c r="G183" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H183" s="1">
         <v>0.25</v>
@@ -9023,7 +9023,7 @@
         <v>83-91</v>
       </c>
       <c r="G184" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H184" s="1">
         <v>0.125</v>
@@ -9070,7 +9070,7 @@
         <v>83-91</v>
       </c>
       <c r="G185" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H185" s="1">
         <v>0.125</v>
@@ -9117,7 +9117,7 @@
         <v>83-91</v>
       </c>
       <c r="G186" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H186" s="1">
         <v>0.2</v>
@@ -9164,7 +9164,7 @@
         <v>87-95</v>
       </c>
       <c r="G187" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H187" s="1">
         <v>0.15</v>
@@ -9211,7 +9211,7 @@
         <v>87-95</v>
       </c>
       <c r="G188" t="str">
-        <v>51-56</v>
+        <v>53-58</v>
       </c>
       <c r="H188" s="1">
         <v>0.15</v>

</xml_diff>